<commit_message>
Remove Redundant pre Nexus 5 Routines
Specifically, these routines are the Asset Hierarchy "Location" Processing routines
</commit_message>
<xml_diff>
--- a/ExcelEventing/EventingTest.xlsx
+++ b/ExcelEventing/EventingTest.xlsx
@@ -8,25 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\Code\Office Macros\InspectorMike Excel Addin\ExcelEventing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5728E099-56CE-4210-B2F4-0A0AFD93B55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A1992E-B94F-4933-803A-1494EA359DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29655" yWindow="-1320" windowWidth="21600" windowHeight="12735" activeTab="1" xr2:uid="{DC716FF6-A397-4893-91C8-FBC114D07AAC}"/>
+    <workbookView xWindow="29475" yWindow="-420" windowWidth="21600" windowHeight="12735" activeTab="2" xr2:uid="{DC716FF6-A397-4893-91C8-FBC114D07AAC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Burial" sheetId="9" r:id="rId1"/>
-    <sheet name="xe.forms" sheetId="2" r:id="rId2"/>
-    <sheet name="xe.lists" sheetId="4" r:id="rId3"/>
-    <sheet name="xe.fields" sheetId="3" r:id="rId4"/>
-    <sheet name="Workpack" sheetId="5" r:id="rId5"/>
-    <sheet name="Component" sheetId="6" r:id="rId6"/>
+    <sheet name="xe.forms" sheetId="2" r:id="rId1"/>
+    <sheet name="xe.lists" sheetId="4" r:id="rId2"/>
+    <sheet name="xe.fields" sheetId="3" r:id="rId3"/>
+    <sheet name="Workpack" sheetId="5" r:id="rId4"/>
+    <sheet name="Component" sheetId="6" r:id="rId5"/>
+    <sheet name="Burial" sheetId="9" r:id="rId6"/>
+    <sheet name="GVI" sheetId="10" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Burial!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Component!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Workpack!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">xe.fields!$A$1:$J$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">xe.forms!$A$1:$D$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">xe.lists!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Burial!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Component!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">GVI!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Workpack!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">xe.fields!$A$1:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">xe.forms!$A$1:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">xe.lists!$A$1:$K$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="85">
   <si>
     <t>FormID</t>
   </si>
@@ -79,21 +81,12 @@
     <t>Workpack</t>
   </si>
   <si>
-    <t>Workpack Entry</t>
-  </si>
-  <si>
     <t>Component</t>
   </si>
   <si>
-    <t>Component Entry</t>
-  </si>
-  <si>
     <t>Burial</t>
   </si>
   <si>
-    <t>Burial Entry</t>
-  </si>
-  <si>
     <t>ControlType</t>
   </si>
   <si>
@@ -106,9 +99,6 @@
     <t>ParentField2</t>
   </si>
   <si>
-    <t>combo</t>
-  </si>
-  <si>
     <t>WorkpackList</t>
   </si>
   <si>
@@ -242,6 +232,69 @@
   </si>
   <si>
     <t>Event</t>
+  </si>
+  <si>
+    <t>GVI</t>
+  </si>
+  <si>
+    <t>Pipeline Burial</t>
+  </si>
+  <si>
+    <t>General Visual Inspection</t>
+  </si>
+  <si>
+    <t>Asset Hierarchy</t>
+  </si>
+  <si>
+    <t>GoodCondition</t>
+  </si>
+  <si>
+    <t>Found in good condition?</t>
+  </si>
+  <si>
+    <t>combobox</t>
+  </si>
+  <si>
+    <t>checkbox</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>Cleaned</t>
+  </si>
+  <si>
+    <t>Any cleaning performed?</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>NVD</t>
+  </si>
+  <si>
+    <t>Log</t>
+  </si>
+  <si>
+    <t>Daily Log</t>
+  </si>
+  <si>
+    <t>"dd MMM yy"</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>y</t>
   </si>
 </sst>
 </file>
@@ -620,76 +673,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BB1050F-FED2-4320-A74F-A47182592FDB}">
-  <sheetPr codeName="Sheet8"/>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E2" s="1">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{8BB1050F-FED2-4320-A74F-A47182592FDB}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5544F1C6-77F4-41A9-AA18-8B60B8273B11}">
   <sheetPr codeName="Sheet2">
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9.140625" style="1"/>
@@ -706,7 +698,7 @@
         <v>5</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -714,50 +706,78 @@
         <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D4" xr:uid="{5544F1C6-77F4-41A9-AA18-8B60B8273B11}"/>
+  <autoFilter ref="A1:D5" xr:uid="{5544F1C6-77F4-41A9-AA18-8B60B8273B11}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73FAE032-2B5D-425E-A71D-D8B2B76B69A0}">
   <sheetPr codeName="Sheet4">
     <tabColor theme="7" tint="0.59999389629810485"/>
@@ -780,48 +800,48 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="H1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>7</v>
@@ -832,13 +852,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>7</v>
@@ -849,19 +869,19 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>7</v>
@@ -872,25 +892,25 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>7</v>
@@ -905,18 +925,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{075F59D9-4A5C-487F-B80C-D42AB058D1D0}">
   <sheetPr codeName="Sheet3">
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -938,7 +959,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>4</v>
@@ -947,30 +968,30 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>8</v>
@@ -978,51 +999,45 @@
       <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>23</v>
-      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>8</v>
@@ -1030,28 +1045,22 @@
       <c r="G4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>8</v>
@@ -1059,77 +1068,71 @@
       <c r="G5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>46</v>
-      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B7" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>8</v>
@@ -1137,28 +1140,37 @@
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="H8" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B9" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1166,22 +1178,31 @@
         <v>14</v>
       </c>
       <c r="B10" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1189,22 +1210,22 @@
         <v>14</v>
       </c>
       <c r="B11" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1212,31 +1233,282 @@
         <v>14</v>
       </c>
       <c r="B12" s="1">
+        <v>6</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="1">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="1">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="1">
         <v>3</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="C15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="1">
+        <v>4</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="I16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="1">
+        <v>5</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" s="1">
+        <v>6</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="1">
+        <v>7</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>7</v>
+      <c r="G19" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="1">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="1">
+        <v>2</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J12" xr:uid="{075F59D9-4A5C-487F-B80C-D42AB058D1D0}"/>
+  <autoFilter ref="A1:J17" xr:uid="{075F59D9-4A5C-487F-B80C-D42AB058D1D0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2A9D6EF-8BED-4FEF-B4E1-3E1316DFA929}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:B3"/>
@@ -1249,26 +1521,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1549,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6997AB8F-AC2C-4837-8CCF-2C656676B197}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:C16"/>
@@ -1291,178 +1563,178 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1473,4 +1745,137 @@
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BB1050F-FED2-4320-A74F-A47182592FDB}">
+  <sheetPr codeName="Sheet8">
+    <tabColor theme="9" tint="0.79998168889431442"/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="1">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{8BB1050F-FED2-4320-A74F-A47182592FDB}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70CAA453-CDE6-4ABE-8800-6DD7F133057C}">
+  <sheetPr>
+    <tabColor theme="9" tint="0.79995117038483843"/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1" xr:uid="{70CAA453-CDE6-4ABE-8800-6DD7F133057C}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ensure only correct routines are exposed to Excel
Added Option Private Module most places
Ensure Private/Public correct
Some refactoring, moving routines to be exposed into correct modules without Option Private Module
Some minor bug fixes
</commit_message>
<xml_diff>
--- a/ExcelEventing/EventingTest.xlsx
+++ b/ExcelEventing/EventingTest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\Code\Office Macros\InspectorMike Excel Addin\ExcelEventing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A1992E-B94F-4933-803A-1494EA359DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1937736D-C5F8-4AE1-9664-381347CFBC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29475" yWindow="-420" windowWidth="21600" windowHeight="12735" activeTab="2" xr2:uid="{DC716FF6-A397-4893-91C8-FBC114D07AAC}"/>
+    <workbookView xWindow="28680" yWindow="-2115" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{DC716FF6-A397-4893-91C8-FBC114D07AAC}"/>
   </bookViews>
   <sheets>
     <sheet name="xe.forms" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Component!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">GVI!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Workpack!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">xe.fields!$A$1:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">xe.fields!$A$1:$J$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">xe.forms!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">xe.lists!$A$1:$K$5</definedName>
   </definedNames>
@@ -40,23 +40,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="87">
   <si>
     <t>FormID</t>
   </si>
   <si>
-    <t>DisplayOrder</t>
-  </si>
-  <si>
-    <t>FieldName</t>
-  </si>
-  <si>
     <t>Label</t>
   </si>
   <si>
-    <t>DataType</t>
-  </si>
-  <si>
     <t>TargetSheet</t>
   </si>
   <si>
@@ -87,18 +78,9 @@
     <t>Burial</t>
   </si>
   <si>
-    <t>ControlType</t>
-  </si>
-  <si>
     <t>ListID</t>
   </si>
   <si>
-    <t>ParentField1</t>
-  </si>
-  <si>
-    <t>ParentField2</t>
-  </si>
-  <si>
     <t>WorkpackList</t>
   </si>
   <si>
@@ -295,6 +277,30 @@
   </si>
   <si>
     <t>y</t>
+  </si>
+  <si>
+    <t>Formid</t>
+  </si>
+  <si>
+    <t>Displayorder</t>
+  </si>
+  <si>
+    <t>Fieldname</t>
+  </si>
+  <si>
+    <t>Controltype</t>
+  </si>
+  <si>
+    <t>Datatype</t>
+  </si>
+  <si>
+    <t>Listid</t>
+  </si>
+  <si>
+    <t>Parentfield1</t>
+  </si>
+  <si>
+    <t>Parentfield2</t>
   </si>
 </sst>
 </file>
@@ -692,83 +698,83 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -800,123 +806,123 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -934,577 +940,578 @@
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>18</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B5" s="1">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B6" s="1">
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1">
         <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1">
         <v>3</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="1">
+        <v>4</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="1">
-        <v>4</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="J10" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B12" s="1">
         <v>6</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B13" s="1">
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B14" s="1">
         <v>2</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B15" s="1">
         <v>3</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="1">
+        <v>4</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="1">
-        <v>4</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B17" s="1">
         <v>5</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1">
         <v>7</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B20" s="1">
         <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B21" s="1">
         <v>2</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B22" s="1">
         <v>3</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J17" xr:uid="{075F59D9-4A5C-487F-B80C-D42AB058D1D0}"/>
+  <autoFilter ref="A1:J22" xr:uid="{075F59D9-4A5C-487F-B80C-D42AB058D1D0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1521,26 +1528,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1563,178 +1570,178 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1766,36 +1773,36 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="E2" s="1">
         <v>5</v>
@@ -1812,7 +1819,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70CAA453-CDE6-4ABE-8800-6DD7F133057C}">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <tabColor theme="9" tint="0.79995117038483843"/>
   </sheetPr>
   <dimension ref="A1:G2"/>
@@ -1830,39 +1837,39 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="E2" s="1" t="b">
         <v>1</v>
@@ -1871,7 +1878,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel Eventing at 1.0
Add Date, Time and DateTime controls
Added intelligent update time code to form
xe.fields validation tool
</commit_message>
<xml_diff>
--- a/ExcelEventing/EventingTest.xlsx
+++ b/ExcelEventing/EventingTest.xlsx
@@ -8,25 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\Code\Office Macros\InspectorMike Excel Addin\ExcelEventing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1937736D-C5F8-4AE1-9664-381347CFBC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C13AAE1-00F9-4FD2-A0F8-8D6B001C2DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2115" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{DC716FF6-A397-4893-91C8-FBC114D07AAC}"/>
+    <workbookView xWindow="28680" yWindow="-2115" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{DC716FF6-A397-4893-91C8-FBC114D07AAC}"/>
   </bookViews>
   <sheets>
     <sheet name="xe.forms" sheetId="2" r:id="rId1"/>
     <sheet name="xe.lists" sheetId="4" r:id="rId2"/>
     <sheet name="xe.fields" sheetId="3" r:id="rId3"/>
     <sheet name="Workpack" sheetId="5" r:id="rId4"/>
-    <sheet name="Component" sheetId="6" r:id="rId5"/>
-    <sheet name="Burial" sheetId="9" r:id="rId6"/>
-    <sheet name="GVI" sheetId="10" r:id="rId7"/>
+    <sheet name="Sheet2" sheetId="12" state="veryHidden" r:id="rId5"/>
+    <sheet name="Component" sheetId="6" r:id="rId6"/>
+    <sheet name="Burial" sheetId="9" r:id="rId7"/>
+    <sheet name="Log" sheetId="11" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Burial!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Component!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">GVI!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Burial!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Component!$A$1:$C$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Log!$A$1:$E$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Workpack!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">xe.fields!$A$1:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">xe.fields!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">xe.forms!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">xe.lists!$A$1:$K$5</definedName>
   </definedNames>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="89">
   <si>
     <t>FormID</t>
   </si>
@@ -252,18 +253,12 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>NVD</t>
-  </si>
-  <si>
     <t>Log</t>
   </si>
   <si>
     <t>Daily Log</t>
   </si>
   <si>
-    <t>"dd MMM yy"</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -276,9 +271,6 @@
     <t>time</t>
   </si>
   <si>
-    <t>y</t>
-  </si>
-  <si>
     <t>Formid</t>
   </si>
   <si>
@@ -301,13 +293,33 @@
   </si>
   <si>
     <t>Parentfield2</t>
+  </si>
+  <si>
+    <t>datetime</t>
+  </si>
+  <si>
+    <t>Start DateTime</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>End DateTime</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,6 +337,19 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
@@ -355,7 +380,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -363,7 +388,40 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -765,16 +823,16 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="C6" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -936,12 +994,12 @@
   <sheetPr codeName="Sheet3">
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -953,34 +1011,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1002,7 +1060,7 @@
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1025,7 +1083,7 @@
       <c r="F3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1048,7 +1106,7 @@
       <c r="F4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1071,7 +1129,7 @@
       <c r="F5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1094,7 +1152,7 @@
       <c r="F6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1117,7 +1175,7 @@
       <c r="F7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H7" s="1" t="s">
@@ -1143,7 +1201,7 @@
       <c r="F8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H8" s="1" t="s">
@@ -1169,7 +1227,7 @@
       <c r="F9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H9" s="1" t="s">
@@ -1198,7 +1256,7 @@
       <c r="F10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H10" s="1" t="s">
@@ -1230,7 +1288,7 @@
       <c r="F11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1253,7 +1311,7 @@
       <c r="F12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1276,7 +1334,7 @@
       <c r="F13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H13" s="1" t="s">
@@ -1302,7 +1360,7 @@
       <c r="F14" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H14" s="1" t="s">
@@ -1328,7 +1386,7 @@
       <c r="F15" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G15" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H15" s="1" t="s">
@@ -1357,7 +1415,7 @@
       <c r="F16" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H16" s="1" t="s">
@@ -1389,7 +1447,7 @@
       <c r="F17" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1412,7 +1470,7 @@
       <c r="F18" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1435,81 +1493,127 @@
       <c r="F19" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B20" s="1">
         <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B21" s="1">
         <v>2</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B22" s="1">
         <v>3</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="1">
+        <v>4</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="1">
+        <v>5</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="G24" s="3" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J22" xr:uid="{075F59D9-4A5C-487F-B80C-D42AB058D1D0}"/>
+  <autoFilter ref="A1:J24" xr:uid="{075F59D9-4A5C-487F-B80C-D42AB058D1D0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1527,26 +1631,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="8" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1557,6 +1661,45 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7194A880-0ED6-415C-812B-ADD3C3500A80}">
+  <sheetPr codeName="Sheet9"/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" style="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6997AB8F-AC2C-4837-8CCF-2C656676B197}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:C16"/>
@@ -1569,192 +1712,188 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="8" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="8" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="8" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="8" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="8" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="8" t="s">
         <v>45</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C8" xr:uid="{6997AB8F-AC2C-4837-8CCF-2C656676B197}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C16">
-      <sortCondition ref="A1:A8"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:C16" xr:uid="{6997AB8F-AC2C-4837-8CCF-2C656676B197}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BB1050F-FED2-4320-A74F-A47182592FDB}">
   <sheetPr codeName="Sheet8">
     <tabColor theme="9" tint="0.79998168889431442"/>
@@ -1762,7 +1901,7 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1771,118 +1910,101 @@
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="8">
         <v>5</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="8">
         <v>25</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{8BB1050F-FED2-4320-A74F-A47182592FDB}"/>
+  <autoFilter ref="A1:F2" xr:uid="{8BB1050F-FED2-4320-A74F-A47182592FDB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70CAA453-CDE6-4ABE-8800-6DD7F133057C}">
-  <sheetPr codeName="Sheet1">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83A0D2A3-434D-44EF-A606-A559F1596B77}">
+  <sheetPr codeName="Sheet7">
     <tabColor theme="9" tint="0.79995117038483843"/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="18.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="2" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>70</v>
-      </c>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="10">
+        <v>46137</v>
+      </c>
+      <c r="B2" s="12">
+        <v>0.58412037037037035</v>
+      </c>
+      <c r="C2" s="14">
+        <v>46137.584108796298</v>
+      </c>
+      <c r="D2" s="14">
+        <v>46137.584120370368</v>
+      </c>
+      <c r="E2" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{70CAA453-CDE6-4ABE-8800-6DD7F133057C}"/>
+  <autoFilter ref="A1:E2" xr:uid="{83A0D2A3-434D-44EF-A606-A559F1596B77}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>